<commit_message>
Atualização automática portal obras
</commit_message>
<xml_diff>
--- a/upload/coordenadas.xlsx
+++ b/upload/coordenadas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F893"/>
+  <dimension ref="A1:F913"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Concluído</t>
+          <t>PRC-29.007/2017-B</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -9084,7 +9084,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Extinto</t>
+          <t>DC-008/2021</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11540,7 +11540,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Rescindido</t>
+          <t>DC-22.016/2020</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -11564,7 +11564,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Rescindido</t>
+          <t>DC-22.016/2020</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -12140,7 +12140,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Rescindido</t>
+          <t>DC-003/2021</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Registro de Preços</t>
+          <t>RP 245/2021</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>Rescindido</t>
+          <t>DC-010/2021</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -20452,7 +20452,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Concluído</t>
+          <t>DER-30.014/2025</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -21820,7 +21820,7 @@
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
@@ -21852,7 +21852,7 @@
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -21884,7 +21884,7 @@
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
@@ -21916,7 +21916,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
@@ -21948,7 +21948,7 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
@@ -21980,7 +21980,7 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
@@ -22012,7 +22012,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DPEI-030/2023</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
@@ -24972,7 +24972,7 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>DOV-002/2021-B</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
@@ -25286,12 +25286,12 @@
       </c>
       <c r="D839" t="inlineStr">
         <is>
-          <t>-17.03493425248546</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E839" t="inlineStr">
         <is>
-          <t>-46.58862620066699</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F839" t="inlineStr">
@@ -25318,12 +25318,12 @@
       </c>
       <c r="D840" t="inlineStr">
         <is>
-          <t>-17.03493425248546</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E840" t="inlineStr">
         <is>
-          <t>-46.58862620066699</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F840" t="inlineStr">
@@ -25345,17 +25345,17 @@
       </c>
       <c r="C841" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D841" t="inlineStr">
         <is>
-          <t>-17.21201508102213</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E841" t="inlineStr">
         <is>
-          <t>-46.687872082284</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F841" t="inlineStr">
@@ -25377,17 +25377,17 @@
       </c>
       <c r="C842" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D842" t="inlineStr">
         <is>
-          <t>-17.21201508102213</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E842" t="inlineStr">
         <is>
-          <t>-46.687872082284</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F842" t="inlineStr">
@@ -25409,17 +25409,17 @@
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>-17.10715545158923</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E843" t="inlineStr">
         <is>
-          <t>-46.62095644999281</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F843" t="inlineStr">
@@ -25441,17 +25441,17 @@
       </c>
       <c r="C844" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D844" t="inlineStr">
         <is>
-          <t>-17.10715545158923</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E844" t="inlineStr">
         <is>
-          <t>-46.62095644999281</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F844" t="inlineStr">
@@ -25463,26 +25463,46 @@
     <row r="845">
       <c r="A845" t="inlineStr">
         <is>
-          <t>DC-9501894/2026</t>
-        </is>
-      </c>
-      <c r="B845" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C845" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D845" t="inlineStr"/>
-      <c r="E845" t="inlineStr"/>
-      <c r="F845" t="inlineStr"/>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>-17.21201508102213</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
-          <t>DC-9518766/2026</t>
-        </is>
-      </c>
-      <c r="B846" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C846" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25490,23 +25510,31 @@
       </c>
       <c r="D846" t="inlineStr">
         <is>
-          <t>-15.483562</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E846" t="inlineStr">
         <is>
-          <t>-44.39677500000001</t>
-        </is>
-      </c>
-      <c r="F846" t="inlineStr"/>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
-          <t>DC-9518766/2026</t>
-        </is>
-      </c>
-      <c r="B847" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C847" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25514,25 +25542,29 @@
       </c>
       <c r="D847" t="inlineStr">
         <is>
-          <t>-15.5007309</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E847" t="inlineStr">
         <is>
-          <t>-44.7624674</t>
-        </is>
-      </c>
-      <c r="F847" t="inlineStr"/>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>DO-009482014/2025-L1</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>9482014</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C848" t="inlineStr">
@@ -25542,29 +25574,29 @@
       </c>
       <c r="D848" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E848" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.687872082284</t>
         </is>
       </c>
       <c r="F848" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="inlineStr">
         <is>
-          <t>DO-009482046/2025-L2</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>9482046</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C849" t="inlineStr">
@@ -25574,29 +25606,29 @@
       </c>
       <c r="D849" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E849" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>DO-009482017/2025-L3</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>9482017</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C850" t="inlineStr">
@@ -25606,29 +25638,29 @@
       </c>
       <c r="D850" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E850" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F850" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C851" t="inlineStr">
@@ -25636,23 +25668,31 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D851" t="inlineStr"/>
-      <c r="E851" t="inlineStr"/>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>-17.10715545158923</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>-46.62095644999281</t>
+        </is>
+      </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>2301617 000003/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C852" t="inlineStr">
@@ -25660,58 +25700,66 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D852" t="inlineStr"/>
-      <c r="E852" t="inlineStr"/>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>-17.10715545158923</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>-46.62095644999281</t>
+        </is>
+      </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>2301617 000003/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="853">
       <c r="A853" t="inlineStr">
         <is>
-          <t>DM-007/2024-A</t>
-        </is>
-      </c>
-      <c r="B853" t="inlineStr"/>
+          <t>DC-9501894/2026</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>9501894</t>
+        </is>
+      </c>
       <c r="C853" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D853" t="inlineStr">
-        <is>
-          <t>-21.1994491</t>
-        </is>
-      </c>
-      <c r="E853" t="inlineStr">
-        <is>
-          <t>-43.7852868</t>
-        </is>
-      </c>
+      <c r="D853" t="inlineStr"/>
+      <c r="E853" t="inlineStr"/>
       <c r="F853" t="inlineStr"/>
     </row>
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B854" t="inlineStr"/>
+          <t>DC-9518766/2026</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>9518766</t>
+        </is>
+      </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>Obra 3</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D854" t="inlineStr">
         <is>
-          <t>-21.27464910003665</t>
+          <t>-15.483562</t>
         </is>
       </c>
       <c r="E854" t="inlineStr">
         <is>
-          <t>-42.91331545001727</t>
+          <t>-44.39677500000001</t>
         </is>
       </c>
       <c r="F854" t="inlineStr"/>
@@ -25719,23 +25767,27 @@
     <row r="855">
       <c r="A855" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B855" t="inlineStr"/>
+          <t>DC-9518766/2026</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>9518766</t>
+        </is>
+      </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>Obra 2</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D855" t="inlineStr">
         <is>
-          <t>-21.23264738347681</t>
+          <t>-15.5007309</t>
         </is>
       </c>
       <c r="E855" t="inlineStr">
         <is>
-          <t>-43.43361939286979</t>
+          <t>-44.7624674</t>
         </is>
       </c>
       <c r="F855" t="inlineStr"/>
@@ -25743,10 +25795,14 @@
     <row r="856">
       <c r="A856" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B856" t="inlineStr"/>
+          <t>DO-009482014/2025-L1</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>9482014</t>
+        </is>
+      </c>
       <c r="C856" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25754,23 +25810,31 @@
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>-21.23528484003703</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E856" t="inlineStr">
         <is>
-          <t>-43.44604111152106</t>
-        </is>
-      </c>
-      <c r="F856" t="inlineStr"/>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
     </row>
     <row r="857">
       <c r="A857" t="inlineStr">
         <is>
-          <t>DC-9519020/2026</t>
-        </is>
-      </c>
-      <c r="B857" t="inlineStr"/>
+          <t>DO-009482046/2025-L2</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>9482046</t>
+        </is>
+      </c>
       <c r="C857" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25778,49 +25842,61 @@
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>-19.6107675</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E857" t="inlineStr">
         <is>
-          <t>-42.64891799999999</t>
-        </is>
-      </c>
-      <c r="F857" t="inlineStr"/>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
     </row>
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>DC-9496643/2026</t>
+          <t>DO-009482017/2025-L3</t>
         </is>
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>9496643</t>
+          <t>9482017</t>
         </is>
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>Obra 2</t>
-        </is>
-      </c>
-      <c r="D858" t="inlineStr"/>
-      <c r="E858" t="inlineStr"/>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>-19.9275586</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>-43.983052</t>
+        </is>
+      </c>
       <c r="F858" t="inlineStr">
         <is>
-          <t>1301606 000002/2025</t>
+          <t>2301901 000001/2025</t>
         </is>
       </c>
     </row>
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t>DC-9496643/2026</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>9496643</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C859" t="inlineStr">
@@ -25828,31 +25904,23 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D859" t="inlineStr">
-        <is>
-          <t>-19.78548575576804</t>
-        </is>
-      </c>
-      <c r="E859" t="inlineStr">
-        <is>
-          <t>-43.9495793253305</t>
-        </is>
-      </c>
+      <c r="D859" t="inlineStr"/>
+      <c r="E859" t="inlineStr"/>
       <c r="F859" t="inlineStr">
         <is>
-          <t>1301606 000002/2025</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>DC-9498666/2026</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B860" t="inlineStr">
         <is>
-          <t>9453556</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C860" t="inlineStr">
@@ -25864,19 +25932,19 @@
       <c r="E860" t="inlineStr"/>
       <c r="F860" t="inlineStr">
         <is>
-          <t>2301520 000041/2025</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr">
         <is>
-          <t>DM-008/2024-A</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>9422064</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C861" t="inlineStr">
@@ -25888,19 +25956,19 @@
       <c r="E861" t="inlineStr"/>
       <c r="F861" t="inlineStr">
         <is>
-          <t>2301762 000036/2023</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>DM-011/2024-A</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>9421657</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C862" t="inlineStr">
@@ -25908,31 +25976,23 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D862" t="inlineStr">
-        <is>
-          <t>-17.335013</t>
-        </is>
-      </c>
-      <c r="E862" t="inlineStr">
-        <is>
-          <t>-44.943418</t>
-        </is>
-      </c>
+      <c r="D862" t="inlineStr"/>
+      <c r="E862" t="inlineStr"/>
       <c r="F862" t="inlineStr">
         <is>
-          <t>2301762 000036/2023</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">
         <is>
-          <t>DM-009/2024-A</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>9422078</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C863" t="inlineStr">
@@ -25944,19 +26004,19 @@
       <c r="E863" t="inlineStr"/>
       <c r="F863" t="inlineStr">
         <is>
-          <t>2301762 000036/2023</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>DM-010/2024-A</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
         <is>
-          <t>9418600</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C864" t="inlineStr">
@@ -25968,17 +26028,21 @@
       <c r="E864" t="inlineStr"/>
       <c r="F864" t="inlineStr">
         <is>
-          <t>2301762 000036/2023</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AMA-9502187/2026</t>
-        </is>
-      </c>
-      <c r="B865" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C865" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25986,15 +26050,23 @@
       </c>
       <c r="D865" t="inlineStr"/>
       <c r="E865" t="inlineStr"/>
-      <c r="F865" t="inlineStr"/>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="866">
       <c r="A866" t="inlineStr">
         <is>
-          <t>DM-9500304/2026</t>
-        </is>
-      </c>
-      <c r="B866" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C866" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26002,15 +26074,23 @@
       </c>
       <c r="D866" t="inlineStr"/>
       <c r="E866" t="inlineStr"/>
-      <c r="F866" t="inlineStr"/>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="867">
       <c r="A867" t="inlineStr">
         <is>
-          <t>DM-9512043/2026</t>
-        </is>
-      </c>
-      <c r="B867" t="inlineStr"/>
+          <t>DM-007/2024-A</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>DM-007/2024-A</t>
+        </is>
+      </c>
       <c r="C867" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26018,12 +26098,12 @@
       </c>
       <c r="D867" t="inlineStr">
         <is>
-          <t>-16.7203311</t>
+          <t>-21.1994491</t>
         </is>
       </c>
       <c r="E867" t="inlineStr">
         <is>
-          <t>-43.8541147</t>
+          <t>-43.7852868</t>
         </is>
       </c>
       <c r="F867" t="inlineStr"/>
@@ -26031,92 +26111,96 @@
     <row r="868">
       <c r="A868" t="inlineStr">
         <is>
-          <t>DC-9497471/2026</t>
+          <t>DC-9515457/2026</t>
         </is>
       </c>
       <c r="B868" t="inlineStr">
         <is>
-          <t>9497471</t>
+          <t>9515457</t>
         </is>
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 3</t>
         </is>
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>-19.747173</t>
+          <t>-21.27464910003665</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>-50.219328</t>
-        </is>
-      </c>
-      <c r="F868" t="inlineStr">
-        <is>
-          <t>1301606 000003/2025</t>
-        </is>
-      </c>
+          <t>-42.91331545001727</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr"/>
     </row>
     <row r="869">
       <c r="A869" t="inlineStr">
         <is>
-          <t>DM-9512044/2026</t>
-        </is>
-      </c>
-      <c r="B869" t="inlineStr"/>
+          <t>DC-9515457/2026</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>9515457</t>
+        </is>
+      </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>Obra 1</t>
-        </is>
-      </c>
-      <c r="D869" t="inlineStr"/>
-      <c r="E869" t="inlineStr"/>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>-21.23264738347681</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>-43.43361939286979</t>
+        </is>
+      </c>
       <c r="F869" t="inlineStr"/>
     </row>
     <row r="870">
       <c r="A870" t="inlineStr">
         <is>
-          <t>DO-001/2021- C</t>
+          <t>DC-9515457/2026</t>
         </is>
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>9275590</t>
+          <t>9515457</t>
         </is>
       </c>
       <c r="C870" t="inlineStr">
         <is>
-          <t>Obra 2</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D870" t="inlineStr">
         <is>
-          <t>-19.928208</t>
+          <t>-21.23528484003703</t>
         </is>
       </c>
       <c r="E870" t="inlineStr">
         <is>
-          <t>-43.983328</t>
-        </is>
-      </c>
-      <c r="F870" t="inlineStr">
-        <is>
-          <t>2301901 000003/2021</t>
-        </is>
-      </c>
+          <t>-43.44604111152106</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr"/>
     </row>
     <row r="871">
       <c r="A871" t="inlineStr">
         <is>
-          <t>DM-017/2024-A</t>
+          <t>DC-9519020/2026</t>
         </is>
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>9424449</t>
+          <t>9519020</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
@@ -26124,55 +26208,51 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D871" t="inlineStr"/>
-      <c r="E871" t="inlineStr"/>
-      <c r="F871" t="inlineStr">
-        <is>
-          <t>2301762 000051/2023</t>
-        </is>
-      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>-19.6107675</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>-42.64891799999999</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr"/>
     </row>
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>DM-014/2024-A</t>
+          <t>DC-9496643/2026</t>
         </is>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>9424302</t>
+          <t>9496643</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>Obra 1</t>
-        </is>
-      </c>
-      <c r="D872" t="inlineStr">
-        <is>
-          <t>-19.8618029</t>
-        </is>
-      </c>
-      <c r="E872" t="inlineStr">
-        <is>
-          <t>-44.5829004</t>
-        </is>
-      </c>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr"/>
+      <c r="E872" t="inlineStr"/>
       <c r="F872" t="inlineStr">
         <is>
-          <t>2301762 000051/2023</t>
+          <t>1301606 000002/2025</t>
         </is>
       </c>
     </row>
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>PRC-29.008/2017-E</t>
+          <t>DC-9496643/2026</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>9149606</t>
+          <t>9496643</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
@@ -26182,29 +26262,29 @@
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>-16.7203311</t>
+          <t>-19.78548575576804</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>-43.8541147</t>
+          <t>-43.9495793253305</t>
         </is>
       </c>
       <c r="F873" t="inlineStr">
         <is>
-          <t>2301901 000001/2017</t>
+          <t>1301606 000002/2025</t>
         </is>
       </c>
     </row>
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>DC-9505062/2026</t>
+          <t>DC-9498666/2026</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>9505062</t>
+          <t>9453556</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
@@ -26212,31 +26292,23 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D874" t="inlineStr">
-        <is>
-          <t>-22.6434039</t>
-        </is>
-      </c>
-      <c r="E874" t="inlineStr">
-        <is>
-          <t>-46.3795013</t>
-        </is>
-      </c>
+      <c r="D874" t="inlineStr"/>
+      <c r="E874" t="inlineStr"/>
       <c r="F874" t="inlineStr">
         <is>
-          <t>2301520 000044/2025</t>
+          <t>2301520 000041/2025</t>
         </is>
       </c>
     </row>
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>DM-9504058/2026</t>
+          <t>DM-008/2024-A</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>9504058</t>
+          <t>9422064</t>
         </is>
       </c>
       <c r="C875" t="inlineStr">
@@ -26244,31 +26316,23 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D875" t="inlineStr">
-        <is>
-          <t>-19.9275586</t>
-        </is>
-      </c>
-      <c r="E875" t="inlineStr">
-        <is>
-          <t>-43.983052</t>
-        </is>
-      </c>
+      <c r="D875" t="inlineStr"/>
+      <c r="E875" t="inlineStr"/>
       <c r="F875" t="inlineStr">
         <is>
-          <t>2301762 000030/2025</t>
+          <t>2301762 000036/2023</t>
         </is>
       </c>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DM-011/2024-A</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9421657</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
@@ -26276,23 +26340,31 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D876" t="inlineStr"/>
-      <c r="E876" t="inlineStr"/>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>-17.335013</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>-44.943418</t>
+        </is>
+      </c>
       <c r="F876" t="inlineStr">
         <is>
-          <t>2301617 000003/2025</t>
+          <t>2301762 000036/2023</t>
         </is>
       </c>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DM-009/2024-A</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9422078</t>
         </is>
       </c>
       <c r="C877" t="inlineStr">
@@ -26304,115 +26376,79 @@
       <c r="E877" t="inlineStr"/>
       <c r="F877" t="inlineStr">
         <is>
-          <t>2301617 000003/2025</t>
+          <t>2301762 000036/2023</t>
         </is>
       </c>
     </row>
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>DC-9501601/2026</t>
+          <t>DM-010/2024-A</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>9501601</t>
+          <t>9418600</t>
         </is>
       </c>
       <c r="C878" t="inlineStr">
         <is>
-          <t>Obra 2</t>
-        </is>
-      </c>
-      <c r="D878" t="inlineStr">
-        <is>
-          <t>-16.11741660736296</t>
-        </is>
-      </c>
-      <c r="E878" t="inlineStr">
-        <is>
-          <t>-45.71048533230583</t>
-        </is>
-      </c>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr"/>
+      <c r="E878" t="inlineStr"/>
       <c r="F878" t="inlineStr">
         <is>
-          <t>2301520 000037/2025</t>
+          <t>2301762 000036/2023</t>
         </is>
       </c>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>DC-9501601/2026</t>
-        </is>
-      </c>
-      <c r="B879" t="inlineStr">
-        <is>
-          <t>9501601</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  AMA-9502187/2026</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr"/>
       <c r="C879" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D879" t="inlineStr">
-        <is>
-          <t>-16.11921421383736</t>
-        </is>
-      </c>
-      <c r="E879" t="inlineStr">
-        <is>
-          <t>-45.58712745575681</t>
-        </is>
-      </c>
-      <c r="F879" t="inlineStr">
-        <is>
-          <t>2301520 000037/2025</t>
-        </is>
-      </c>
+      <c r="D879" t="inlineStr"/>
+      <c r="E879" t="inlineStr"/>
+      <c r="F879" t="inlineStr"/>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>DC-9501601/2026</t>
+          <t>DM-9500304/2026</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>9501601</t>
+          <t>9500304</t>
         </is>
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>Obra 3</t>
-        </is>
-      </c>
-      <c r="D880" t="inlineStr">
-        <is>
-          <t>-16.12119845072</t>
-        </is>
-      </c>
-      <c r="E880" t="inlineStr">
-        <is>
-          <t>-45.6488268407393</t>
-        </is>
-      </c>
-      <c r="F880" t="inlineStr">
-        <is>
-          <t>2301520 000037/2025</t>
-        </is>
-      </c>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr"/>
+      <c r="E880" t="inlineStr"/>
+      <c r="F880" t="inlineStr"/>
     </row>
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>DC-9493529/2026</t>
+          <t>DM-9512043/2026</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>9493529</t>
+          <t>9512043</t>
         </is>
       </c>
       <c r="C881" t="inlineStr">
@@ -26420,23 +26456,27 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D881" t="inlineStr"/>
-      <c r="E881" t="inlineStr"/>
-      <c r="F881" t="inlineStr">
-        <is>
-          <t>2301520 000036/2025</t>
-        </is>
-      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>-16.7203311</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>-43.8541147</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr"/>
     </row>
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>DM-012/2024-A</t>
+          <t>DC-9497471/2026</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>9422079</t>
+          <t>9497471</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
@@ -26444,23 +26484,31 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D882" t="inlineStr"/>
-      <c r="E882" t="inlineStr"/>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>-19.747173</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>-50.219328</t>
+        </is>
+      </c>
       <c r="F882" t="inlineStr">
         <is>
-          <t>2301762 000036/2023</t>
+          <t>1301606 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>DM-9502116/2026</t>
+          <t>DM-9512044/2026</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>9502116</t>
+          <t>9512044</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
@@ -26470,45 +26518,49 @@
       </c>
       <c r="D883" t="inlineStr"/>
       <c r="E883" t="inlineStr"/>
-      <c r="F883" t="inlineStr">
-        <is>
-          <t>2301762 000026/2025</t>
-        </is>
-      </c>
+      <c r="F883" t="inlineStr"/>
     </row>
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>DM-018/2024-A</t>
+          <t>DO-001/2021- C</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>9424304</t>
+          <t>9275590</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>Obra 1</t>
-        </is>
-      </c>
-      <c r="D884" t="inlineStr"/>
-      <c r="E884" t="inlineStr"/>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>-19.928208</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>-43.983328</t>
+        </is>
+      </c>
       <c r="F884" t="inlineStr">
         <is>
-          <t>2301762 000051/2023</t>
+          <t>2301901 000003/2021</t>
         </is>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>DM-016/2024-A</t>
+          <t>DM-017/2024-A</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>9424337</t>
+          <t>9424449</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
@@ -26527,12 +26579,12 @@
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>DM-020/2024-A</t>
+          <t>DM-014/2024-A</t>
         </is>
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>9427674</t>
+          <t>9424302</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
@@ -26542,12 +26594,12 @@
       </c>
       <c r="D886" t="inlineStr">
         <is>
-          <t>-17.8518635</t>
+          <t>-19.8618029</t>
         </is>
       </c>
       <c r="E886" t="inlineStr">
         <is>
-          <t>-41.5076927</t>
+          <t>-44.5829004</t>
         </is>
       </c>
       <c r="F886" t="inlineStr">
@@ -26559,12 +26611,12 @@
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>DM-022/2024-A</t>
+          <t>PRC-29.008/2017-E</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>9427765</t>
+          <t>9149606</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
@@ -26574,91 +26626,143 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>-20.6829764</t>
+          <t>-16.7203311</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
         <is>
-          <t>-44.8232506</t>
+          <t>-43.8541147</t>
         </is>
       </c>
       <c r="F887" t="inlineStr">
         <is>
-          <t>2301762 000051/2023</t>
+          <t>2301901 000001/2017</t>
         </is>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>DC-9511902/2026</t>
-        </is>
-      </c>
-      <c r="B888" t="inlineStr"/>
+          <t>DC-9505062/2026</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>9505062</t>
+        </is>
+      </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>Obra 4</t>
-        </is>
-      </c>
-      <c r="D888" t="inlineStr"/>
-      <c r="E888" t="inlineStr"/>
-      <c r="F888" t="inlineStr"/>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>-22.6434039</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>-46.3795013</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>2301520 000044/2025</t>
+        </is>
+      </c>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t>DC-9511902/2026</t>
-        </is>
-      </c>
-      <c r="B889" t="inlineStr"/>
+          <t>DM-9504058/2026</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>9504058</t>
+        </is>
+      </c>
       <c r="C889" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D889" t="inlineStr"/>
-      <c r="E889" t="inlineStr"/>
-      <c r="F889" t="inlineStr"/>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>-19.9275586</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>2301762 000030/2025</t>
+        </is>
+      </c>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
         <is>
-          <t>DC-9511902/2026</t>
-        </is>
-      </c>
-      <c r="B890" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>Obra 3</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D890" t="inlineStr"/>
       <c r="E890" t="inlineStr"/>
-      <c r="F890" t="inlineStr"/>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="891">
       <c r="A891" t="inlineStr">
         <is>
-          <t>DC-9511902/2026</t>
-        </is>
-      </c>
-      <c r="B891" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>Obra 2</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D891" t="inlineStr"/>
       <c r="E891" t="inlineStr"/>
-      <c r="F891" t="inlineStr"/>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>DM-9519034/2026</t>
-        </is>
-      </c>
-      <c r="B892" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C892" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26666,31 +26770,539 @@
       </c>
       <c r="D892" t="inlineStr"/>
       <c r="E892" t="inlineStr"/>
-      <c r="F892" t="inlineStr"/>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr"/>
+      <c r="E893" t="inlineStr"/>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr"/>
+      <c r="E894" t="inlineStr"/>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr"/>
+      <c r="E895" t="inlineStr"/>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr"/>
+      <c r="E896" t="inlineStr"/>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr"/>
+      <c r="E897" t="inlineStr"/>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>DC-9501601/2026</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>9501601</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>-16.11741660736296</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>-45.71048533230583</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>2301520 000037/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>DC-9501601/2026</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>9501601</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>-16.11921421383736</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>-45.58712745575681</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>2301520 000037/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>DC-9501601/2026</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>9501601</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Obra 3</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>-16.12119845072</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>-45.6488268407393</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>2301520 000037/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>DC-9493529/2026</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>9493529</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr"/>
+      <c r="E901" t="inlineStr"/>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>2301520 000036/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>DM-012/2024-A</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>9422079</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr"/>
+      <c r="E902" t="inlineStr"/>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>2301762 000036/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>DM-9502116/2026</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>9502116</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr"/>
+      <c r="E903" t="inlineStr"/>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>2301762 000026/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>DM-018/2024-A</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>9424304</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr"/>
+      <c r="E904" t="inlineStr"/>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>2301762 000051/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>DM-016/2024-A</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>9424337</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr"/>
+      <c r="E905" t="inlineStr"/>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>2301762 000051/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>DM-020/2024-A</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>9427674</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>-17.8518635</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>-41.5076927</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>2301762 000051/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>DM-022/2024-A</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>9427765</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>-20.6829764</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>-44.8232506</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>2301762 000051/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>DC-9511902/2026</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Obra 4</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr"/>
+      <c r="E908" t="inlineStr"/>
+      <c r="F908" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>DC-9511902/2026</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr"/>
+      <c r="E909" t="inlineStr"/>
+      <c r="F909" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>DC-9511902/2026</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Obra 3</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr"/>
+      <c r="E910" t="inlineStr"/>
+      <c r="F910" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>DC-9511902/2026</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr"/>
+      <c r="E911" t="inlineStr"/>
+      <c r="F911" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>DM-9519034/2026</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>9519034</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr"/>
+      <c r="E912" t="inlineStr"/>
+      <c r="F912" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
           <t>DC-9519017/2026</t>
         </is>
       </c>
-      <c r="B893" t="inlineStr"/>
-      <c r="C893" t="inlineStr">
-        <is>
-          <t>Obra 1</t>
-        </is>
-      </c>
-      <c r="D893" t="inlineStr">
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>9519017</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
         <is>
           <t>-18.46005275010656</t>
         </is>
       </c>
-      <c r="E893" t="inlineStr">
+      <c r="E913" t="inlineStr">
         <is>
           <t>-48.18218127247928</t>
         </is>
       </c>
-      <c r="F893" t="inlineStr"/>
+      <c r="F913" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>